<commit_message>
test case enhnacmenst[pepsico],bug fixes in xpath, page file,test file
</commit_message>
<xml_diff>
--- a/output/xpath_generator/xpath_details.xlsx
+++ b/output/xpath_generator/xpath_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -938,6 +938,890 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//form//input[@id='login-button']  </t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//div[contains(@class, 'form-group')]//input[@id='login-button']  </t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//*[@id='login-button']//parent::div  </t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>//*[@id='login-button']//preceding-sibling::*</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Login Button (input#login-button)  </t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>//*//input[@name='login-button']</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>//div[contains(@class, 'submit-button')]//input[@id='login-button']</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>user-name</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@name='user-name']  </t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>### Add to Cart: Test AllTheThings T-Shirt (Red) (button with id="add-to-cart-test.allthethings()-t-shirt-(red)")</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[text()='Add to cart']  </t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>### Open Menu</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[@id='react-burger-menu-btn']  </t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>tes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[contains(@class, 'btn_action')]  </t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>### Open Menu Button</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[text()='Open Menu']  </t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>### Open Menu (button with id=react-burger-menu-btn)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[@text()='Open Menu']  </t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Open Menu</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>//button[text()='Open Menu']</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>### Open Menu</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[@id='react-burger-menu-btn']  </t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Login Button (input)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>//ancestor::form//input[@id='login-button']</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[contains(@name, 'login-button')]  </t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[parent::*[@class='form-actions']]  </t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>### Element: input[id='login-button']</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>//input[@id='login-button' and (@class='submit-button btn_action' or @name='login-button')]</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>User Name Input</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='user-name']  </t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>User Name Input Field (id=user-name)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>/input[@id='user-name']</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>User Name Input Field:</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>//input[@id='user-name']</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>User-Name Input Field</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='user-name']  </t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Password Input Field</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='password']  </t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='login-button']  </t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>### Element: Close button</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[@class='close']  </t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>### Element: CONTINUE button</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[@id='continue-button']  </t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>### Element: zip</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='zip']  </t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>### Element: Select state</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[contains(@text, 'Select state')]  </t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>### Element: city</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='city']  </t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>### Element: addressLine2Id</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='addressLine2Id']  </t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>### Element: address</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='address']  </t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>### Element: phoneNumber</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='phoneNumber']  </t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>### Element: ssn</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='ssn']  </t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>### Element: dob</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='dob']  </t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>### Element: lastName</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='lastName']  </t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>### Element: firstNameId</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='firstNameId']  </t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Equfix_place_an_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>### firstNameId</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='firstNameId']  </t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>### lastName</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='lastName']  </t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>### dob</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='dob']  </t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>### ssn</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='ssn']  </t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>### phoneNumber</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='phoneNumber']  </t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>### address</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='address']  </t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>### addressLine2Id</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='addressLine2Id']  </t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>### city</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='city']  </t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>### zip</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='zip']  </t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>### efx-dropdown-label-796908</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[starts-with(@id, 'efx-dropdown-label')]  </t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>### continue-button</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//button[@id='continue-button']  </t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Equfixplaceanalert</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>User Name Input</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='user-name']  </t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>User Name Input</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@name='user-name']  </t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>User Name Input</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='user-name' and @name='user-name']  </t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Password Input</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='password']  </t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Login Button</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='login-button']  </t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test case category enhancements, bug fixes,prompt generation,chibot implemntation
</commit_message>
<xml_diff>
--- a/output/xpath_generator/xpath_details.xlsx
+++ b/output/xpath_generator/xpath_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">//input[@id='user-name']  </t>
+          <t xml:space="preserve">//input[@name='user-name']  </t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">//input[@name='user-name']  </t>
+          <t xml:space="preserve">//input[@id='user-name' and @name='user-name']  </t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1774,12 +1774,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>User Name Input</t>
+          <t>User Name (input)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">//input[@id='user-name' and @name='user-name']  </t>
+          <t xml:space="preserve">//input[@id='user-name']  </t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1791,7 +1791,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Password Input</t>
+          <t>Password (input)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1808,7 +1808,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Login Button</t>
+          <t>Login Button (input)</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1819,6 +1819,57 @@
       <c r="C82" t="inlineStr">
         <is>
           <t>Sauce_demo_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Element: a.btn.gcs-btn.gcs-btn--secondary.gcs-btn--pill.gcs-btn--border.mt-3.mx-1.PLACE AN ALERT  </t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//a[contains(@class, 'gcs-btn') and contains(text(), 'PLACE AN ALERT')]  </t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Equ_home_page</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>firstNameId</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='firstNameId']  </t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>equ_place_on_alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>lastName</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">//input[@id='lastName']  </t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>equ_place_on_alert</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
IQEA_refined_version - full local changes sync
- Updated Self_healing_web_application: features, xpath details, DOM details, dom_collector.js, validated xpath
- Updated action_new_xpath_subway.py, llm_test.py, utilities/Utilities_Xpath.py
- Updated output: xpath_details.xlsx, Action_collection assets
- Added mobile recordings (April & May 2026), screenshots, test cases, generated scripts
- Added output/allure-results from latest runs
- Removed stale root allure-results artifacts

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/xpath_generator/xpath_details.xlsx
+++ b/output/xpath_generator/xpath_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C208"/>
+  <dimension ref="A1:C211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3964,6 +3964,57 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Input (id='user-name')</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> //input[@id='user-name']</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>test_xapth</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Input (id='password')</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> //input[@id='password']</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>test_xapth</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>user-name (id='user-name')</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> //input[@id='user-name']</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>login_page</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
pbi validator enhancements slicer and action recording enahnacements
</commit_message>
<xml_diff>
--- a/output/xpath_generator/xpath_details.xlsx
+++ b/output/xpath_generator/xpath_details.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C214"/>
+  <dimension ref="A1:C216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4066,6 +4066,40 @@
         </is>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Input @id='user-name'</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>//input[@id='user-name']</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>sauce_logi</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Hierarchical combined XPaths</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>//input[@id='login-button']/preceding-sibling::input[@id='password']</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>sauce_logi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chat and new UI for IQEA
</commit_message>
<xml_diff>
--- a/output/xpath_generator/xpath_details.xlsx
+++ b/output/xpath_generator/xpath_details.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C216"/>
+  <dimension ref="A1:C218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4100,6 +4100,40 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>user-name (id='user-name')</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> //input[@id='login-button']</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>test_login</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>user-name (id='user-name')</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> //input[@id='password']/preceding::input[@id='user-name']</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>test_login</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>